<commit_message>
Add partner API TCs, fix SA/portal UI TCs after FE changes, update bug tracker
- New API TCs: deal stats, forgot password, portal bank accounts/catalogue/clients/commissions/plans, partner team, SA attributions/commissions summary/deals list/link tenant/partner update/user unlock

- UI: register wizard domain inputs match the new rule; SA directory Pending filter + deactivate reason; My Apps removed from shell sections

- Drop be_gap for fixed bugs (UI-001/003/006/008); BUG-UI-010 for /directory mobile overflow

- Selftest: marker-vs-tracker compares OPEN bugs only
</commit_message>
<xml_diff>
--- a/docs/blazeup/Bug_Tracker.xlsx
+++ b/docs/blazeup/Bug_Tracker.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -110,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -118,7 +124,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,15 +145,28 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="1" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -513,25 +532,25 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17.14785714285714" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="12" min="2" max="2"/>
-    <col width="46.005" bestFit="1" customWidth="1" style="11" min="3" max="3"/>
-    <col width="12.005" bestFit="1" customWidth="1" style="11" min="4" max="4"/>
-    <col width="16.005" bestFit="1" customWidth="1" style="11" min="5" max="5"/>
-    <col width="9.005000000000001" bestFit="1" customWidth="1" style="11" min="6" max="6"/>
-    <col width="8.005000000000001" bestFit="1" customWidth="1" style="11" min="7" max="7"/>
-    <col width="10.005" bestFit="1" customWidth="1" style="11" min="8" max="8"/>
-    <col width="40.005" bestFit="1" customWidth="1" style="11" min="9" max="9"/>
-    <col width="38.005" bestFit="1" customWidth="1" style="11" min="10" max="10"/>
-    <col width="34.005" bestFit="1" customWidth="1" style="11" min="11" max="11"/>
-    <col width="42.005" bestFit="1" customWidth="1" style="11" min="12" max="12"/>
-    <col width="12.005" bestFit="1" customWidth="1" style="11" min="13" max="13"/>
-    <col width="11.005" bestFit="1" customWidth="1" style="11" min="14" max="14"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="11" min="15" max="15"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="11" min="16" max="16"/>
+    <col width="17.14785714285714" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="16" min="2" max="2"/>
+    <col width="46.005" bestFit="1" customWidth="1" style="15" min="3" max="3"/>
+    <col width="12.005" bestFit="1" customWidth="1" style="15" min="4" max="4"/>
+    <col width="16.005" bestFit="1" customWidth="1" style="15" min="5" max="5"/>
+    <col width="9.005000000000001" bestFit="1" customWidth="1" style="15" min="6" max="6"/>
+    <col width="8.005000000000001" bestFit="1" customWidth="1" style="15" min="7" max="7"/>
+    <col width="10.005" bestFit="1" customWidth="1" style="15" min="8" max="8"/>
+    <col width="40.005" bestFit="1" customWidth="1" style="15" min="9" max="9"/>
+    <col width="38.005" bestFit="1" customWidth="1" style="15" min="10" max="10"/>
+    <col width="34.005" bestFit="1" customWidth="1" style="15" min="11" max="11"/>
+    <col width="42.005" bestFit="1" customWidth="1" style="15" min="12" max="12"/>
+    <col width="12.005" bestFit="1" customWidth="1" style="15" min="13" max="13"/>
+    <col width="11.005" bestFit="1" customWidth="1" style="15" min="14" max="14"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="15" min="15" max="15"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="15" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customFormat="1" customHeight="1" s="1">
@@ -2079,700 +2098,1713 @@
       <c r="P22" s="7" t="n"/>
     </row>
     <row r="23" ht="58.5" customHeight="1">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>BUG-API-021</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="15" t="inlineStr">
         <is>
           <t>(no TC yet — DELETE partner is never asserted)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>PARTNER_ACCOUNT_MANAGEMENT</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="15" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="15" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" s="15" t="inlineStr">
         <is>
           <t>Soft delete is INTENTIONAL (confirmed by BE) — but a deleted partner and a suspended one both end up with status='suspended', so no client can tell them apart. The business status 'suspended' has effectively lost its meaning, and QA has no way to remove test data.</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J23" s="15" t="inlineStr">
         <is>
           <t>Keep the soft delete. Add a way to DISTINGUISH the two states — e.g. a read-only deletedAt / isDeleted field, or an optional filter on GET /v1/sa/partners. No behaviour change needed and SA can still see every partner. Separately: a supported way for QA to purge its own test data (maintenance endpoint, or an agreed manual DB cleanup).</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K23" s="15" t="inlineStr">
         <is>
           <t>DELETE returns 200 {"message":"Partner deleted successfully"}; the record stays, status flips pending/active -&gt; 'suspended' and internalNotes -&gt; 'Deleted by SA'. That free-text note is the ONLY signal separating a deleted partner from a genuinely suspended one. Measured on stgsa 2026-08-10: 2371 of 2416 partners are 'suspended', and 2369 of those carry 'Deleted by SA' — so only 2 are real suspensions. Volume is also growing: 1808 partners on 2026-08-06 -&gt; 2416 on 2026-08-10 (+608 in 4 days), and nothing can remove them.</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L23" s="15" t="inlineStr">
         <is>
           <t>Probe on stgsa 2026-08-06: create partner -&gt; DELETE (200) -&gt; GET /v1/sa/partners?search=&lt;name&gt; still returns it at +0s/+3s/+10s with status='suspended', internalNotes='Deleted by SA'. Reproduced from a UI run: 'CLEANUP LEAK: DELETE partner ... returned HTTP 200 but the record is STILL listed'.</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M23" s="15" t="inlineStr">
         <is>
           <t>QA (review)</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="N23" s="15" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="O23" s="15" t="n"/>
+      <c r="P23" s="15" t="inlineStr">
         <is>
           <t>BE DESIGN CONFIRMED (Khoa Nguyen, 2026-08-10): partners are never hard-deleted on purpose — SA must see every partner, and the status has to be revertible. So this is NOT a request to hard delete; the remaining ask is only a field that separates 'deleted' from 'suspended'. | Impact on automation: created_resources cleanup receives 200 and reports success while removing nothing — that is how ~2.4k QA-AUTO partners accumulated unnoticed. utils/ui_cleanup.py and utils/cleanup_staging.py now re-read the record after DELETE and report CLEANUP LEAK instead of trusting the status code. | Impact on testing: PARTNER_UI_SA_PARTNER_MODULE_016 (reactivate) needs a genuinely Suspended partner and only 2 candidates exist among 2371 rows. | Also missing, tracked here for now: no DELETE for deals, and no delete/revoke for partner-users (only certifications), so data created by PARTNER_UI_MY_PIPELINE_005 and PARTNER_UI_PARTNER_TEAM_001 cannot be cleaned by any route. | Open question back to Product: should 'application declined' and 'active partner suspended' really share one status too? deactivate serves both.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18.75" customHeight="1">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="9" t="n"/>
-      <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="7" t="n"/>
-      <c r="I24" s="7" t="n"/>
-      <c r="J24" s="7" t="n"/>
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
-      <c r="M24" s="7" t="n"/>
-      <c r="N24" s="7" t="n"/>
-      <c r="O24" s="7" t="n"/>
-      <c r="P24" s="7" t="n"/>
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-022</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>2061401</v>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_TEAM_001</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_TEAM</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I24" s="15" t="inlineStr">
+        <is>
+          <t>partner team directory - invited member appears in list and detail.</t>
+        </is>
+      </c>
+      <c r="J24" s="15" t="inlineStr">
+        <is>
+          <t>partner team directory - invited member appears in list and detail.</t>
+        </is>
+      </c>
+      <c r="K24" s="15" t="inlineStr">
+        <is>
+          <t>FAIL | [6/6] Read the session user by id → must return THAT user (259ms) -- AssertionError: GET /directory/users/{userId} ignored the path parameter: asked for 6aaa783b5a1d688484cf3045, got 6aaa783f5a1d688484cf3059 (team.qa.auto+aaron35-aa19222eed3b@</t>
+        </is>
+      </c>
+      <c r="L24" s="15" t="inlineStr">
+        <is>
+          <t>FAIL | [6/6] Read the session user by id → must return THAT user (259ms) -- AssertionError: GET /directory/users/{userId} ignored the path parameter: asked for 6aaa783b5a1d688484cf3045, got 6aaa783f5a1d688484cf3059 (team.qa.auto+aaron35-aa19222eed3b@mailinator.com). A ghost id and a malformed id ret</t>
+        </is>
+      </c>
+      <c r="M24" s="15" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N24" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O24" s="15" t="n"/>
+      <c r="P24" s="15" t="n"/>
     </row>
     <row r="25" ht="18.75" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-023</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>2061403</v>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_TEAM_003</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_TEAM</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H25" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I25" s="15" t="inlineStr">
+        <is>
+          <t>team member deals and commissions - own records, scoped.</t>
+        </is>
+      </c>
+      <c r="J25" s="15" t="inlineStr">
+        <is>
+          <t>team member deals and commissions - own records, scoped.</t>
+        </is>
+      </c>
+      <c r="K25" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FAIL | [6/7] The rollup must DISCRIMINATE between members (547ms) -- AssertionError: GET /directory/users/{userId}/deals ignores the path parameter: the member 6aab91e1b8ca8e4baea2a4ca registered NO deals, yet asking for it returns the same 1 row(s) </t>
+        </is>
+      </c>
+      <c r="L25" s="15" t="inlineStr">
+        <is>
+          <t>FAIL | [6/7] The rollup must DISCRIMINATE between members (547ms) -- AssertionError: GET /directory/users/{userId}/deals ignores the path parameter: the member 6aab91e1b8ca8e4baea2a4ca registered NO deals, yet asking for it returns the same 1 row(s) as the session user who registered them. A ghost u</t>
+        </is>
+      </c>
+      <c r="M25" s="15" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N25" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="O25" s="15" t="n"/>
+      <c r="P25" s="15" t="n"/>
+    </row>
+    <row r="26" ht="18.75" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-024</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>2060124</v>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_ACCOUNT_MANAGEMENT_024</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_ACCOUNT_MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I26" s="15" t="inlineStr">
+        <is>
+          <t>PATCH /v1/sa/partners/:id accepts fields UpdatePartnerDto does not expose. _id -&gt; HTTP 500 leaking the MongoDB error; code and status are silently written. Writing status moves a PENDING partner straight to active.</t>
+        </is>
+      </c>
+      <c r="J26" s="15" t="inlineStr">
+        <is>
+          <t>A field outside UpdatePartnerDto is ignored or refused with 400 — never a 5xx, never a write. status must change only through POST /partners/:id/approve|deactivate, so the 3-stage approval FSM (PRD §12.1 B3: SA Review -&gt; Legal Countersign -&gt; SA Final Approval) cannot be skipped. Error bodies must not expose the storage engine.</t>
+        </is>
+      </c>
+      <c r="K26" s="15" t="inlineStr">
+        <is>
+          <t>PATCH {"_id": "&lt;ghost&gt;"} -&gt; 500 "Plan executor error during findAndModify :: caused by :: Performing an update on the path '_id' would modify the immutable field '_id'". PATCH {"code": "QA-HACKED"} -&gt; 200 and the partner code is overwritten. PATCH {"status": "active"} -&gt; 200 and a pending partner becomes active without approve.</t>
+        </is>
+      </c>
+      <c r="L26" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_ACCOUNT_MANAGEMENT_024 step [5/5], staging 2026-09-17, BE v26 @ 0b35609. Each field sent on its own so the failing one is named. The positive TC _023 passes: the 6 declared fields persist and a repeat PATCH is idempotent.</t>
+        </is>
+      </c>
+      <c r="M26" s="15" t="inlineStr">
+        <is>
+          <t>QA (automation)</t>
+        </is>
+      </c>
+      <c r="N26" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="O26" s="15" t="n"/>
+      <c r="P26" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS BE CONFIRMATION on the status part: is writing status through PATCH intended for SA, or an FSM bypass? The _id 500 and the writable code are defects either way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18.75" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-025</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>2060236</v>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_DEAL_REGISTRATION_PIPELINE_036</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>DEAL_REGISTRATION_PIPELINE</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I27" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/sa/deals: limit=0 and page=abc are accepted and the endpoint returns the ENTIRE result set in one page (1406 deals). limit=-1 is correctly refused with 400.</t>
+        </is>
+      </c>
+      <c r="J27" s="15" t="inlineStr">
+        <is>
+          <t>Any nonsensical pagination value is refused with 400, the same way limit=-1 already is. A page size must never resolve to unbounded.</t>
+        </is>
+      </c>
+      <c r="K27" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/sa/deals?limit=0  -&gt; 200, data[] holds 1406 rows. GET /v1/sa/deals?page=abc -&gt; 200, data[] holds 1406 rows. GET /v1/sa/deals?limit=-1 -&gt; 400 "Invalid pagination: limit must be a positive integer".</t>
+        </is>
+      </c>
+      <c r="L27" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_DEAL_REGISTRATION_PIPELINE_036 step [3/4], staging 2026-09-21, BE v26 @ 0b35609. The positive TC _035 passes: partnerId, status and dealType all narrow correctly and limit=1 caps the page.</t>
+        </is>
+      </c>
+      <c r="M27" s="15" t="inlineStr">
+        <is>
+          <t>QA (automation)</t>
+        </is>
+      </c>
+      <c r="N27" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="O27" s="15" t="n"/>
+      <c r="P27" s="15" t="inlineStr">
+        <is>
+          <t>Impact is a full-table dump per request, not just a validation gap — worth checking whether other list endpoints share the same pagination guard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18.75" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-026</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>2060908</v>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_PORTAL_008</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_PORTAL</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H28" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I28" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/partner/portal/modules: groupByCategory=true returns rows that are only {"_id": "undefined"}, and no pagination value is validated (limit=-1, limit=0 and page=abc all answer 200 with the whole catalogue).</t>
+        </is>
+      </c>
+      <c r="J28" s="15" t="inlineStr">
+        <is>
+          <t>groupByCategory=true returns usable groups (a category name and its modules). Nonsensical pagination is refused with 400 — GET /v1/sa/deals already refuses limit=-1, so the service knows how to do this.</t>
+        </is>
+      </c>
+      <c r="K28" s="15" t="inlineStr">
+        <is>
+          <t>GET /portal/modules?groupByCategory=true -&gt; 200, total=23, data[] holds 10 objects each exactly {"_id": "undefined"} — the literal JS string "undefined", no name, no members. GET /portal/modules?limit=-1 -&gt; 200 (1 row); ?limit=0 and ?page=abc -&gt; 200 with all 23 rows.</t>
+        </is>
+      </c>
+      <c r="L28" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_PORTAL_008 steps [4/5] and [5/5], staging 2026-09-21, BE v26 @ 0b35609. The positive TC _007 passes: the plain catalogue, the name filter, and both team-certification filters all narrow correctly.</t>
+        </is>
+      </c>
+      <c r="M28" s="15" t="inlineStr">
+        <is>
+          <t>QA (automation)</t>
+        </is>
+      </c>
+      <c r="N28" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="O28" s="15" t="n"/>
+      <c r="P28" s="15" t="inlineStr">
+        <is>
+          <t>The pagination half is the same class as BUG-API-025 on /v1/sa/deals but a different endpoint and stricter: /sa/deals at least refuses limit=-1, this one refuses nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18.75" customHeight="1">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-027</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>2061510</v>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_CLIENT_HEALTH_MSP_010</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>CLIENT_HEALTH_MSP</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I29" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/partner/portal/clients: limit=0 and page=abc are not validated and answer 200. limit=-1 IS refused with 400, so the guard exists on this very endpoint and simply misses the other two values.</t>
+        </is>
+      </c>
+      <c r="J29" s="15" t="inlineStr">
+        <is>
+          <t>A nonsensical page size or page number is refused with 400, consistently with limit=-1 on the same endpoint and with GET /v1/sa/deals.</t>
+        </is>
+      </c>
+      <c r="K29" s="15" t="inlineStr">
+        <is>
+          <t>GET /portal/clients?limit=-1 -&gt; 400 (correct). ?limit=0 -&gt; 200. ?page=abc -&gt; 200. Both returned 0 rows, but only because the caller had no clients: the value was accepted rather than rejected, so the row count proves nothing about the guard.</t>
+        </is>
+      </c>
+      <c r="L29" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_CLIENT_HEALTH_MSP_010 step [4/4], staging 2026-09-21, BE v26 @ 0b35609. The rest of the TC passes: a ghost attribution id and a malformed id are both refused with 400 and neither refusal leaks client row fields. The positive TC _001 passes in full, including JWT scoping (a partnerId in the query does not widen the result).</t>
+        </is>
+      </c>
+      <c r="M29" s="15" t="inlineStr">
+        <is>
+          <t>QA (automation)</t>
+        </is>
+      </c>
+      <c r="N29" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="O29" s="15" t="n"/>
+      <c r="P29" s="15" t="inlineStr">
+        <is>
+          <t>Third endpoint with the same root cause, after BUG-API-025 (/v1/sa/deals) and BUG-API-026 (/v1/partner/portal/modules) — worth ONE shared fix rather than three. Severity is lower here only because this list is empty on staging (no attribution is reachable, G2); the same miss on /sa/deals dumps 1406 rows in a single page, so the impact returns as soon as a partner owns clients.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18.75" customHeight="1">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-028</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="n">
+        <v>2061613</v>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_TENANT_PROVISIONING_ATTRIBUTION_013</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>TENANT_PROVISIONING_ATTRIBUTION</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G30" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H30" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I30" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/sa/partner-attributions: limit=0 and page=abc are not validated and answer 200 with the whole ledger. limit=-1 IS refused with 400, so the guard exists on this very endpoint and misses the other two values.</t>
+        </is>
+      </c>
+      <c r="J30" s="15" t="inlineStr">
+        <is>
+          <t>A nonsensical page size or page number is refused with 400, consistently with limit=-1 on the same endpoint.</t>
+        </is>
+      </c>
+      <c r="K30" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/sa/partner-attributions?limit=-1 -&gt; 400 "Invalid pagination: limit must be a positive integer" (correct). ?limit=0 -&gt; 200 with all 10 rows. ?page=abc -&gt; 200 with all 10 rows. Unlike the portal twin this list is NOT empty, so the caller receives the entire SA-wide ledger in one page.</t>
+        </is>
+      </c>
+      <c r="L30" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_TENANT_PROVISIONING_ATTRIBUTION_013 step [4/4], staging 2026-09-23, BE v26. The rest of the TC passes: status/clientLifecycleState outside the enum -&gt; 400 listing the allowed values, malformed partnerId and malformed attribution id -&gt; 400, ghost partnerId -&gt; 200 empty, ghost attribution id -&gt; 400. The positive TC _012 passes in full (10 rows across 6 distinct partners, partnerId filter narrows 10 -&gt; 1, detail route returns the requested row).</t>
+        </is>
+      </c>
+      <c r="M30" s="15" t="inlineStr">
+        <is>
+          <t>QA (automation)</t>
+        </is>
+      </c>
+      <c r="N30" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="O30" s="15" t="n"/>
+      <c r="P30" s="15" t="inlineStr">
+        <is>
+          <t>FOURTH endpoint with the identical root cause: BUG-API-025 (/v1/sa/deals), BUG-API-026 (/v1/partner/portal/modules), BUG-API-027 (/v1/partner/portal/clients), now this one. Every instance refuses limit=-1 and accepts limit=0 and page=abc, which points at one shared pagination validator rather than four separate misses. Recommend BE fix it once at that layer and close all four together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18.75" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-029</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n">
+        <v>2060910</v>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_PORTAL_010</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_PORTAL</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H31" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I31" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/partner/portal/plans/{planId}: the path parameter named planId is the only value it will NOT accept. The route matches on the mongo _id; a plan's own planId slug answers 400 'Invalid id'.</t>
+        </is>
+      </c>
+      <c r="J31" s="15" t="inlineStr">
+        <is>
+          <t>The parameter documented by the route's own @ApiParam as a 'Kebab-case plan key, e.g. pro-annual' resolves the plan. Either the implementation should query { planId: &lt;slug&gt; }, or the route, @ApiParam and the service docstring should all say _id.</t>
+        </is>
+      </c>
+      <c r="K31" s="15" t="inlineStr">
+        <is>
+          <t>GET /portal/plans returns rows carrying both _id and planId. GET /portal/plans/6aa76eab1e7d8bcb2279dd3f (the _id) -&gt; 200 with the plan. GET /portal/plans/full-modules-ss (that same row's planId) -&gt; 400 "Invalid id: 'full-modules-ss'". partner-lookup.service.ts getPlanByPlanId queries { _id: planId, status: PUBLISHED } while its docstring says 'Fetches a published billing plan by its planId slug'.</t>
+        </is>
+      </c>
+      <c r="L31" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_PORTAL_010 step [2/4], staging 2026-09-23, BE v26. The rest of the pair passes: _009 verifies the catalogue is published standard editions only with unique ids/slugs and an exact detail match by _id; _010 confirms a ghost key -&gt; 404 naming it and 'not-a-plan'/'%20'/'null' -&gt; 400. | PROBE 2026-09-28 (live): GET /v1/partner/portal/plans/{_id=6aa76eab1e7d8bcb2279dd3f} -&gt; 200 (returns the plan); GET /v1/partner/portal/plans/{planId='full-modules-ss'} -&gt; 400 'Invalid id: full-modules-ss'. Same plan object carries BOTH _id (ObjectId) and planId (slug); the catalogue returns planId as a field and the route is declared plans/:planId with @ApiParam=slug, but the service queries {_id: param} so only the ObjectId is accepted. Confirmed BE contract bug (NOT test-data): the param named planId is the one value it rejects.</t>
+        </is>
+      </c>
+      <c r="M31" s="15" t="inlineStr">
+        <is>
+          <t>QA (automation)</t>
+        </is>
+      </c>
+      <c r="N31" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="O31" s="15" t="n"/>
+      <c r="P31" s="15" t="inlineStr">
+        <is>
+          <t>Contract-level, not a crash: the deal-registration form works because it passes _id. The cost is that any client written from the OpenAPI spec fails 100% of the time, and the naming actively misleads - a reader has no way to tell from the route that planId means _id. Low fix cost either way; BE only needs to decide which side is authoritative. NOT related to the pagination family (BUG-API-025/026/027/028). | FIX (BE): either (a) accept the slug on plans/:planId (query {planId: param} or fall back), matching the param name + OpenAPI docs [expected per spec]; or (b) rename param to :id + document ObjectId and have callers use _id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18.75" customHeight="1">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-030</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="n">
+        <v>2060324</v>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_COMMISSIONS_PAYOUTS_024</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr">
+        <is>
+          <t>COMMISSIONS_PAYOUTS</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H32" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I32" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/partner/portal/commissions: limit=0 and page=abc are not validated and answer 200. limit=-1 IS refused with 400 on the same endpoint.</t>
+        </is>
+      </c>
+      <c r="J32" s="15" t="inlineStr">
+        <is>
+          <t>A nonsensical page size or page number is refused with 400, consistently with limit=-1 on the same endpoint.</t>
+        </is>
+      </c>
+      <c r="K32" s="15" t="inlineStr">
+        <is>
+          <t>?limit=-1 -&gt; 400 'Invalid pagination: limit must be a positive integer' (correct). ?limit=0 -&gt; 200. ?page=abc -&gt; 200. Both returned 0 rows, but only because no commission exists anywhere on staging (G1): the value was accepted rather than rejected, so the row count proves nothing about the guard.</t>
+        </is>
+      </c>
+      <c r="L32" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_COMMISSIONS_PAYOUTS_024 step [3/3], staging 2026-09-24, BE v26. The rest of the pair passes: status='bogus' -&gt; 400 listing all eight statuses; the positive TC _020 passes in full (envelope, all 8 status values accepted, ledger agrees with its summary, a partnerId in the query does not widen the JWT scope).</t>
+        </is>
+      </c>
+      <c r="M32" s="15" t="inlineStr">
+        <is>
+          <t>QA (automation)</t>
+        </is>
+      </c>
+      <c r="N32" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O32" s="15" t="n"/>
+      <c r="P32" s="15" t="inlineStr">
+        <is>
+          <t>FIFTH endpoint with the identical root cause: BUG-API-025 (/v1/sa/deals), 026 (/v1/partner/portal/modules), 027 (/v1/partner/portal/clients), 028 (/v1/sa/partner-attributions), now this one. Every instance refuses limit=-1 and accepts limit=0 and page=abc. Five independent misses of the same two values is not plausible - this is one shared pagination validator, and one fix at that layer should close all five together. Filed separately only so each failing TC has its own traceable row; recommend BE treat 025/026/027/028/030 as a single defect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18.75" customHeight="1">
+      <c r="A33" s="7" t="n"/>
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="n"/>
+      <c r="H33" s="7" t="n"/>
+      <c r="I33" s="7" t="n"/>
+      <c r="J33" s="7" t="n"/>
+      <c r="K33" s="7" t="n"/>
+      <c r="L33" s="7" t="n"/>
+      <c r="M33" s="7" t="n"/>
+      <c r="N33" s="7" t="n"/>
+      <c r="O33" s="7" t="n"/>
+      <c r="P33" s="7" t="n"/>
+    </row>
+    <row r="34" ht="18.75" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="B25" s="10" t="n"/>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="6" t="n"/>
-      <c r="J25" s="6" t="n"/>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
-      <c r="M25" s="6" t="n"/>
-      <c r="N25" s="6" t="n"/>
-      <c r="O25" s="6" t="n"/>
-      <c r="P25" s="6" t="n"/>
-    </row>
-    <row r="26" ht="18.75" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="6" t="n"/>
+      <c r="I34" s="6" t="n"/>
+      <c r="J34" s="6" t="n"/>
+      <c r="K34" s="6" t="n"/>
+      <c r="L34" s="6" t="n"/>
+      <c r="M34" s="6" t="n"/>
+      <c r="N34" s="6" t="n"/>
+      <c r="O34" s="6" t="n"/>
+      <c r="P34" s="6" t="n"/>
+    </row>
+    <row r="35" ht="18.75" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>BUG-UI-001</t>
         </is>
       </c>
-      <c r="B26" s="9" t="n">
+      <c r="B35" s="9" t="n">
         <v>12060101</v>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>PARTNER_UI_PARTNER_PORTAL_SHELL_001</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>PARTNER_PORTAL_SHELL</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
         <is>
           <t>every primary nav page loads via URL (no MFE error).</t>
         </is>
       </c>
-      <c r="J26" s="7" t="inlineStr">
+      <c r="J35" s="7" t="inlineStr">
         <is>
           <t>every primary nav page loads via URL (no MFE error).</t>
         </is>
       </c>
-      <c r="K26" s="7" t="n"/>
-      <c r="L26" s="7" t="inlineStr">
+      <c r="K35" s="7" t="n"/>
+      <c r="L35" s="7" t="inlineStr">
         <is>
           <t>Page [apps] FAILED - Partner Portal section 'apps' rendered its shell but the CONTENT failed to load: banner 'Failed to load' is visible in &lt;main&gt;. Data-fetch/backend issue for this page — confirm with BE.</t>
         </is>
       </c>
-      <c r="M26" s="7" t="inlineStr">
+      <c r="M35" s="7" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N26" s="7" t="inlineStr">
+      <c r="N35" s="7" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="O26" s="7" t="n"/>
-      <c r="P26" s="7" t="n"/>
-    </row>
-    <row r="27" ht="18.75" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="O35" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P35" s="7" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-09-30 — no longer applicable: the 'My Apps' page was REMOVED from the partner portal (no nav item; /apps renders a 404 page). 'apps' dropped from the test; PARTNER_UI_PARTNER_PORTAL_SHELL_001 now PASSES 5/5, be_gap removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18.75" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>BUG-UI-002</t>
         </is>
       </c>
-      <c r="B27" s="9" t="n">
+      <c r="B36" s="9" t="n">
         <v>12060102</v>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>PARTNER_UI_PARTNER_PORTAL_SHELL_002</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
         <is>
           <t>PARTNER_PORTAL_SHELL</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="inlineStr">
         <is>
           <t>portal stays usable at mobile width (no h-overflow, nav reachable).</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
+      <c r="J36" s="7" t="inlineStr">
         <is>
           <t>portal stays usable at mobile width (no h-overflow, nav reachable).</t>
         </is>
       </c>
-      <c r="K27" s="7" t="inlineStr">
+      <c r="K36" s="7" t="inlineStr">
         <is>
           <t>Page [deals] FAILED - 'deals' overflows the mobile viewport by 162px (content does not fit 375px → responsive-layout defect; confirm with FE)</t>
         </is>
       </c>
-      <c r="L27" s="7" t="inlineStr">
+      <c r="L36" s="7" t="inlineStr">
         <is>
           <t>Page [deals] FAILED - 'deals' overflows the mobile viewport by 162px (content does not fit 375px → responsive-layout defect; confirm with FE)</t>
         </is>
       </c>
-      <c r="M27" s="7" t="inlineStr">
+      <c r="M36" s="7" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N27" s="7" t="inlineStr">
+      <c r="N36" s="7" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="O27" s="7" t="n"/>
-      <c r="P27" s="7" t="n"/>
-    </row>
-    <row r="28" ht="18.75" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="O36" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P36" s="7" t="inlineStr">
+        <is>
+          <t>FIXED — re-verified 2026-09-30: /deals no longer overflows at 375px (was +162px). My Apps page removed from the portal. TC 12060102 still fails, but ONLY on /directory — a distinct defect logged as BUG-UI-010.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18.75" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>BUG-UI-003</t>
         </is>
       </c>
-      <c r="B28" s="9" t="n">
+      <c r="B37" s="9" t="n">
         <v>12060203</v>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>PARTNER_UI_MY_PIPELINE_003</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>MY_PIPELINE</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I28" s="7" t="inlineStr">
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
         <is>
           <t>an invalid domain must be rejected with a format error.</t>
         </is>
       </c>
-      <c r="J28" s="7" t="inlineStr">
+      <c r="J37" s="7" t="inlineStr">
         <is>
           <t>an invalid domain must be rejected with a format error.</t>
         </is>
       </c>
-      <c r="K28" s="7" t="inlineStr">
+      <c r="K37" s="7" t="inlineStr">
         <is>
           <t>FAIL | [1/1] Each malformed domain must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts invalid domain(s) ["'@@@' (field kept '@@@', Next enabled, not flagged)", "'ab cd' (field kept 'ab cd', Next enabled, not flagged)</t>
         </is>
       </c>
-      <c r="L28" s="7" t="inlineStr">
+      <c r="L37" s="7" t="inlineStr">
         <is>
           <t>FAIL | [1/1] Each malformed domain must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts invalid domain(s) ["'@@@' (field kept '@@@', Next enabled, not flagged)", "'ab cd' (field kept 'ab cd', Next enabled, not flagged)", "'notadomain' (field kept 'notadomain', Next en</t>
         </is>
       </c>
-      <c r="M28" s="7" t="inlineStr">
+      <c r="M37" s="7" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N28" s="7" t="inlineStr">
+      <c r="N37" s="7" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="O28" s="7" t="n"/>
-      <c r="P28" s="7" t="n"/>
-    </row>
-    <row r="29" ht="18.75" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="O37" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P37" s="7" t="inlineStr">
+        <is>
+          <t>FIXED — re-verified 2026-09-30: the Domain field now validates ('Use letters, numbers, and hyphens only — no dots or symbols, e.g. my-company'). Test inputs corrected: 'notadomain' removed (VALID under the rule) and replaced with 'acme.com'. PARTNER_UI_MY_PIPELINE_003 PASSES, be_gap removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18.75" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>BUG-UI-004</t>
         </is>
       </c>
-      <c r="B29" s="9" t="n">
+      <c r="B38" s="9" t="n">
         <v>12060207</v>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>PARTNER_UI_MY_PIPELINE_007</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>MY_PIPELINE</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H38" s="7" t="inlineStr">
         <is>
           <t>CLOSE
 CLOSE
 CLOSE</t>
         </is>
       </c>
-      <c r="I29" s="7" t="inlineStr">
+      <c r="I38" s="7" t="inlineStr">
         <is>
           <t>a malformed contact email must be rejected with a format error.</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
+      <c r="J38" s="7" t="inlineStr">
         <is>
           <t>a malformed contact email must be rejected with a format error.</t>
         </is>
       </c>
-      <c r="K29" s="7" t="inlineStr">
+      <c r="K38" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">FAIL | [1/1] Each malformed email must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts malformed email(s) ["'notanemail' (field kept 'notanemail', Next enabled, not flagged)", "'abc@' (field kept 'abc@', Next enabled, </t>
         </is>
       </c>
-      <c r="L29" s="7" t="inlineStr">
+      <c r="L38" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">FAIL | [1/1] Each malformed email must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts malformed email(s) ["'notanemail' (field kept 'notanemail', Next enabled, not flagged)", "'abc@' (field kept 'abc@', Next enabled, not flagged)", "'abc@x' (field kept 'abc@x', Next </t>
         </is>
       </c>
-      <c r="M29" s="7" t="inlineStr">
+      <c r="M38" s="7" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N29" s="7" t="inlineStr">
+      <c r="N38" s="7" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="O29" s="7" t="n"/>
-      <c r="P29" s="7" t="n"/>
-    </row>
-    <row r="30" ht="18.75" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="O38" s="7" t="n"/>
+      <c r="P38" s="7" t="n"/>
+    </row>
+    <row r="39" ht="18.75" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>BUG-UI-005</t>
         </is>
       </c>
-      <c r="B30" s="9" t="n">
+      <c r="B39" s="9" t="n">
         <v>12060507</v>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>PARTNER_UI_SA_PARTNER_MODULE_007</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
         <is>
           <t>SA_PARTNER_MODULE</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>CLOSE</t>
         </is>
       </c>
-      <c r="I30" s="7" t="inlineStr">
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>SA Deal Approval Queue (/partners/deals): deal-list API consistently returns "Server Error - Invalid id: pro-v1" instead of the deals.</t>
         </is>
       </c>
-      <c r="J30" s="7" t="inlineStr">
+      <c r="J39" s="7" t="inlineStr">
         <is>
           <t>GET deal-list for /partners/deals returns the deals (200); the queue table shows deal rows. No "Invalid id" error.</t>
         </is>
       </c>
-      <c r="K30" s="7" t="inlineStr">
+      <c r="K39" s="7" t="inlineStr">
         <is>
           <t>The deal-list fetch consistently returns "Server Error - Invalid id: pro-v1"; the UI shows "No Data Found" and no deal rows load (partners DO have open deals).</t>
         </is>
       </c>
-      <c r="L30" s="7" t="inlineStr">
+      <c r="L39" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">FAIL | [3/3] The Pending Approval + Conflicts queues load without a server error (3161ms) -- AssertionError: the deal approval queues must load their deals, but the deal-list fetch fails with a backend error on: ['Pending Approval: "Server Error Invalid id: \'pro-v1\' Server Error Invalid id: \'"', </t>
         </is>
       </c>
-      <c r="M30" s="7" t="inlineStr">
+      <c r="M39" s="7" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N30" s="7" t="inlineStr">
+      <c r="N39" s="7" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="O30" s="7" t="inlineStr">
+      <c r="O39" s="7" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="P30" s="7" t="inlineStr">
+      <c r="P39" s="7" t="inlineStr">
         <is>
           <t>FIXED — re-verified 2026-08-10: PARTNER_UI_SA_PARTNER_MODULE_007 now PASSES (15.3s, log: 'CHECK deals load -&gt; OK (no server error)'). The deal-list fetch no longer returns "Invalid id: 'pro-v1'". be_gap marker removed from the test and the registry re-synced, so this TC is back inside the merge gate. | Root cause = contract drift: a plan-slug "pro-v1" (string) is used where the API expects a Mongo _id (24-hex), so deal-list id validation fails. CONSISTENT, not intermittent (updated 2026-08-05): earlier "lucky PASS" runs were a TEST race - the assertion ran before the async deal-list error painted; the test now waits for the fetch to settle and fails deterministically. UI test 12060507 renders fine (shell/filters/headers OK); this step reflects the BE defect. Fix BE so deal-list never returns Invalid id: pro-v1.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18.75" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
+    <row r="40" ht="18.75" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>BUG-UI-006</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n">
+      <c r="B40" s="9" t="n">
         <v>12060511</v>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>PARTNER_UI_SA_PARTNER_MODULE_011</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>SA_PARTNER_MODULE</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>the SA partner-programme analytics dashboard.</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>the SA partner-programme analytics dashboard.</t>
+        </is>
+      </c>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [3/3] The analytics data loads without a server error (44ms) -- AssertionError: the analytics dashboard must load its data, but a query fails with a backend error: 'Server Error limit must not be greater than 100 Server Error Invalid p'. The d</t>
+        </is>
+      </c>
+      <c r="L40" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [3/3] The analytics data loads without a server error (44ms) -- AssertionError: the analytics dashboard must load its data, but a query fails with a backend error: 'Server Error limit must not be greater than 100 Server Error Invalid p'. The dashboard shell renders but a paginated analytics q</t>
+        </is>
+      </c>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N40" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="O40" s="7" t="n"/>
+      <c r="P40" s="7" t="n"/>
+    </row>
+    <row r="41" ht="18.75" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>BUG-UI-007</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>12060405</v>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>PARTNER_UI_DASHBOARD_005</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>DASHBOARD</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
-        <is>
-          <t>the SA partner-programme analytics dashboard.</t>
-        </is>
-      </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>the SA partner-programme analytics dashboard.</t>
-        </is>
-      </c>
-      <c r="K31" s="7" t="inlineStr">
-        <is>
-          <t>FAIL | [3/3] The analytics data loads without a server error (44ms) -- AssertionError: the analytics dashboard must load its data, but a query fails with a backend error: 'Server Error limit must not be greater than 100 Server Error Invalid p'. The d</t>
-        </is>
-      </c>
-      <c r="L31" s="7" t="inlineStr">
-        <is>
-          <t>FAIL | [3/3] The analytics data loads without a server error (44ms) -- AssertionError: the analytics dashboard must load its data, but a query fails with a backend error: 'Server Error limit must not be greater than 100 Server Error Invalid p'. The dashboard shell renders but a paginated analytics q</t>
-        </is>
-      </c>
-      <c r="M31" s="7" t="inlineStr">
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>tier-qualification math (T12M ARR threshold + next-tier delta).</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>tier-qualification math (T12M ARR threshold + next-tier delta).</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [2/3] Next-tier T12M ARR threshold target + remaining delta are shown (0ms) -- AssertionError: the next-tier T12M ARR threshold target and remaining delta must be shown in Tier Progress, but only current tier/ARR/deal-count are rendered (panel</t>
+        </is>
+      </c>
+      <c r="L41" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [2/3] Next-tier T12M ARR threshold target + remaining delta are shown (0ms) -- AssertionError: the next-tier T12M ARR threshold target and remaining delta must be shown in Tier Progress, but only current tier/ARR/deal-count are rendered (panel='Tier &amp; Performance SELECT T12M ARR USD 0 Tier Pr</t>
+        </is>
+      </c>
+      <c r="M41" s="7" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N31" s="7" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="O31" s="7" t="n"/>
-      <c r="P31" s="7" t="n"/>
-    </row>
-    <row r="32" ht="18.75" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>BUG-UI-007</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="n">
-        <v>12060405</v>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>PARTNER_UI_DASHBOARD_005</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>DASHBOARD</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="N41" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="O41" s="7" t="n"/>
+      <c r="P41" s="7" t="n"/>
+    </row>
+    <row r="42" ht="18.75" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>BUG-UI-008</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>12060515</v>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>PARTNER_UI_SA_PARTNER_MODULE_015</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>SA_PARTNER_MODULE</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G42" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>suspend (deactivate) an active partner.</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>SA can suspend an Active partner from Partner Detail -&gt; Partner actions -&gt; Deactivate: partner transitions to Suspended/Inactive and loses portal access.</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>Deactivate fails. The "Deactivate Partner" confirm dialog collects NO reason, so the FE calls the deactivate API without one; BE returns 400 Server Error ("reason should not be empty / reason must be a string / reason must be &lt;= 2000 characters"). Partner stays Active. No SA can suspend a partner via the UI.</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [2/2] The partner is suspended and no error is shown (0ms) -- AssertionError: Deactivate failed — the BE rejected the request: 'Failed to deactivate partner Server Error reason must be shorter than or equal to 2000 charactersreason should not be emptyreason must be a string Partner approved Q</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N42" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="O42" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P42" s="7" t="inlineStr">
+        <is>
+          <t>FIXED — re-verified 2026-09-30: the Deactivate Partner dialog now has a required Reason textarea (Deactivate disabled until filled); the request succeeds and the partner becomes Suspended. PARTNER_UI_SA_PARTNER_MODULE_015 PASSES, be_gap removed. Unblocks _016 (reactivate). | FE&lt;-&gt;BE contract mismatch. Fix options: (a) add a required Reason textarea to the Deactivate dialog and send it, or (b) make reason optional on the deactivate API. Repro: onboard partner -&gt; Approve -&gt; Partner actions -&gt; Deactivate -&gt; Confirm. Blocks SA_PARTNER_MODULE_016 (reactivate) too. TC marked be_gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18.75" customHeight="1">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>BUG-UI-009</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="n">
+        <v>12060201</v>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_UI_MY_PIPELINE_001</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>MY_PIPELINE</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="I43" s="15" t="inlineStr">
+        <is>
+          <t>Register-a-Deal wizard: Country dropdown is empty ('No options') on Chrome/Chromium (works on Edge). The wizard's countries lookup is sent WITHOUT an Authorization header -&gt; 401, so no country can be selected and a deal cannot be registered.</t>
+        </is>
+      </c>
+      <c r="J43" s="15" t="inlineStr">
+        <is>
+          <t>On every browser (incl. Chrome) the Country dropdown lists countries; partner completes Step 1 and registers a deal.</t>
+        </is>
+      </c>
+      <c r="K43" s="15" t="inlineStr">
+        <is>
+          <t>On Chrome/Chromium (manual AND automation), GET /sa-partners-api/v1/partner/portal/countries is sent with NO Authorization header -&gt; 401 -&gt; dropdown shows 'No options' -&gt; Step 1 cannot be completed. On Edge (manual) the same request carries the bearer token -&gt; 200 -&gt; options load.</t>
+        </is>
+      </c>
+      <c r="L43" s="15" t="inlineStr">
+        <is>
+          <t>countries request hasAuth=false -&gt; 401 on Chromium (Playwright) and manual Chrome; 200 on manual Edge. Shell /partner/auth/refresh + /auth/me return 200, so the shell is authenticated but the token is not attached to the MFE's countries call. Manual repro: Chrome FAIL / Edge PASS.</t>
+        </is>
+      </c>
+      <c r="M43" s="15" t="inlineStr">
+        <is>
+          <t>tam.do@terralogic.com</t>
+        </is>
+      </c>
+      <c r="N43" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O43" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P43" s="15" t="inlineStr">
+        <is>
+          <t>FIXED — verified manually by QA on 2026-09-30 (ticket BLAZ7-5-27 PV VALIDATION → CLOSED): Country dropdown loads on Chrome. | Browser-specific (Chrome/Chromium FAIL, Edge PASS) at BOTH manual and automation level. Affects all 11 register-wizard TCs: 12060201-12060208, 12060211-12060213 (automation runs on Chromium -&gt; all fail). Leading hypothesis for FE: Chrome's stricter storage-partitioning / third-party-context defaults block the deals micro-frontend (partnerDealsApp, which has its own token-store bundle) from reading the auth token (pp_refresh_token in sessionStorage) -&gt; token not attached to the countries request. FE to verify how partnerDealsApp obtains/attaches the access token on Chrome. NOTE: AI triage mislabels these as [FLAKY] (Locator.click-timeout heuristic) - they are deterministic, not flaky.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18.75" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-031</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="n">
+        <v>2061402</v>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_TEAM_002</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_TEAM</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H44" s="15" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr">
-        <is>
-          <t>tier-qualification math (T12M ARR threshold + next-tier delta).</t>
-        </is>
-      </c>
-      <c r="J32" s="7" t="inlineStr">
-        <is>
-          <t>tier-qualification math (T12M ARR threshold + next-tier delta).</t>
-        </is>
-      </c>
-      <c r="K32" s="7" t="inlineStr">
-        <is>
-          <t>FAIL | [2/3] Next-tier T12M ARR threshold target + remaining delta are shown (0ms) -- AssertionError: the next-tier T12M ARR threshold target and remaining delta must be shown in Tier Progress, but only current tier/ARR/deal-count are rendered (panel</t>
-        </is>
-      </c>
-      <c r="L32" s="7" t="inlineStr">
-        <is>
-          <t>FAIL | [2/3] Next-tier T12M ARR threshold target + remaining delta are shown (0ms) -- AssertionError: the next-tier T12M ARR threshold target and remaining delta must be shown in Tier Progress, but only current tier/ARR/deal-count are rendered (panel='Tier &amp; Performance SELECT T12M ARR USD 0 Tier Pr</t>
-        </is>
-      </c>
-      <c r="M32" s="7" t="inlineStr">
+      <c r="I44" s="15" t="inlineStr">
+        <is>
+          <t>Partner team directory read-by-id ignores the path parameter: a ghost (well-formed, absent) userId is not rejected, and a malformed userId is not rejected.</t>
+        </is>
+      </c>
+      <c r="J44" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/partner/directory/users/{userId}: a ghost (well-formed but non-existent) userId -&gt; 404 not found; a malformed userId -&gt; 400 invalid id.</t>
+        </is>
+      </c>
+      <c r="K44" s="15" t="inlineStr">
+        <is>
+          <t>ghost userId 000000000000000000000000 -&gt; HTTP 200 returning a DIFFERENT user (userId=6aba0a4b...); malformed userId 'not-an-id' -&gt; HTTP 200. The path parameter is ignored, so a caller reading a member it never asked for gets no error at all.</t>
+        </is>
+      </c>
+      <c r="L44" s="15" t="inlineStr">
+        <is>
+          <t>FAIL test_partner_api_partner_team_002 (run 2026-09-28): 'Validation gaps on /v1/partner/directory/users: ghost userId 000...000 returned HTTP 200 with userId=6aba0a4b... instead of 404; malformed userId not-an-id returned HTTP 200 instead of 400.'</t>
+        </is>
+      </c>
+      <c r="M44" s="15" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N32" s="7" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="O32" s="7" t="n"/>
-      <c r="P32" s="7" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>BUG-UI-008</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="n">
-        <v>12060515</v>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>PARTNER_UI_SA_PARTNER_MODULE_015</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>SA_PARTNER_MODULE</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="N44" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O44" s="15" t="n"/>
+      <c r="P44" s="15" t="inlineStr">
+        <is>
+          <t>Negative counterpart of BUG-API-022 (2061401) - SAME root cause: GET /directory/users/{userId} ignores the path param. Fix together with BUG-API-022/023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="204" customHeight="1">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-032</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="n">
+        <v>2061404</v>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_TEAM_004</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_TEAM</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G45" s="15" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H45" s="15" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
-        <is>
-          <t>suspend (deactivate) an active partner.</t>
-        </is>
-      </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>SA can suspend an Active partner from Partner Detail -&gt; Partner actions -&gt; Deactivate: partner transitions to Suspended/Inactive and loses portal access.</t>
-        </is>
-      </c>
-      <c r="K33" s="7" t="inlineStr">
-        <is>
-          <t>Deactivate fails. The "Deactivate Partner" confirm dialog collects NO reason, so the FE calls the deactivate API without one; BE returns 400 Server Error ("reason should not be empty / reason must be a string / reason must be &lt;= 2000 characters"). Partner stays Active. No SA can suspend a partner via the UI.</t>
-        </is>
-      </c>
-      <c r="L33" s="7" t="inlineStr">
-        <is>
-          <t>FAIL | [2/2] The partner is suspended and no error is shown (0ms) -- AssertionError: Deactivate failed — the BE rejected the request: 'Failed to deactivate partner Server Error reason must be shorter than or equal to 2000 charactersreason should not be emptyreason must be a string Partner approved Q</t>
-        </is>
-      </c>
-      <c r="M33" s="7" t="inlineStr">
+      <c r="I45" s="15" t="inlineStr">
+        <is>
+          <t>Team member deals/commissions read ignores the path parameter: a ghost/malformed userId is not rejected (reads as a member with no records).</t>
+        </is>
+      </c>
+      <c r="J45" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/partner/directory/users/{userId}/{deals,commissions}: a ghost userId -&gt; 404 not found; a malformed userId -&gt; 400 invalid id.</t>
+        </is>
+      </c>
+      <c r="K45" s="15" t="inlineStr">
+        <is>
+          <t>ghost userId -&gt; HTTP 200 with 0 rows (expected 404); malformed userId -&gt; HTTP 200 with 0 rows (expected 400). Path param ignored -&gt; a non-existent member reads as one that simply has no records; the same call returns ANOTHER member's deals when there ARE any (see BUG-API-023 / _003) = cross-member data disclosure risk.</t>
+        </is>
+      </c>
+      <c r="L45" s="15" t="inlineStr">
+        <is>
+          <t>FAIL test_partner_api_partner_team_004 (run 2026-09-28): 'Validation gaps on /v1/partner/directory/users/{userId}/{deals,commissions}: ghost userId answered 200 with 0 rows, expected 404 - the path parameter is ignored (BUG-API-023); malformed userId answered 200 with 0 rows, expected 400.'</t>
+        </is>
+      </c>
+      <c r="M45" s="15" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N33" s="7" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="O33" s="7" t="n"/>
-      <c r="P33" s="7" t="inlineStr">
-        <is>
-          <t>FE&lt;-&gt;BE contract mismatch. Fix options: (a) add a required Reason textarea to the Deactivate dialog and send it, or (b) make reason optional on the deactivate API. Repro: onboard partner -&gt; Approve -&gt; Partner actions -&gt; Deactivate -&gt; Confirm. Blocks SA_PARTNER_MODULE_016 (reactivate) too. TC marked be_gap.</t>
+      <c r="N45" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O45" s="15" t="n"/>
+      <c r="P45" s="15" t="inlineStr">
+        <is>
+          <t>Negative counterpart of BUG-API-023 (2061403) - SAME root cause: GET /directory/users/{userId}/{deals,commissions} ignores the path param. Fix together with BUG-API-022/023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BUG-UI-010</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="n">
+        <v>12060102</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PARTNER_UI_PARTNER_PORTAL_SHELL_002</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>PARTNER_PORTAL_SHELL</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Partner Portal /directory overflows horizontally at mobile width (375px): the 'Invite User' button and the member table do not fit, so the whole page scrolls sideways.</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>At 375×812 the Directory page fits the viewport (horizontal overflow ≤ 5px); the member table scrolls inside its own container if it is wider than the screen.</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>The page overflows by +93px (scrollWidth 468 vs 375): the 'Invite User' button sticks out 93px and the member table (MEMBER / ROLE / STATUS / LAST LOGIN) is ~607px wider than the viewport with no overflow-x wrapper.</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Page [directory] FAILED - 'directory' overflows the mobile viewport by 93px (content does not fit 375px → responsive-layout defect; confirm with FE) | probe: documentElement.scrollWidth=468 vs clientWidth=375; 'Invite User' button right edge +93px; member &lt;table&gt; right edge +607px (no overflow-x container)</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Distinct from BUG-UI-002 (Deals overflow, now fixed) — same TC, different page/cause, kept as its own bug. Other pages (dashboard/deals/commissions/resources) fit. Fix: wrap the member table in an overflow-x:auto container and let the header action bar wrap/stack on small screens.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Allure: mark soft-failed steps red; fix TC 2060122 (re-grant = renewal), close BUG-API-001
</commit_message>
<xml_diff>
--- a/docs/blazeup/Bug_Tracker.xlsx
+++ b/docs/blazeup/Bug_Tracker.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>CLOSE</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -726,8 +726,16 @@
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="O3" s="7" t="n"/>
-      <c r="P3" s="7" t="n"/>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="P3" s="7" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-10-01 — NOT A BUG (works as designed, confirmed by BE / Khoa Nguyen on PPM-BUG-01): re-grant is a RENEWAL — the active cert is revoked (revokeReason=superseded_by_renewal) and one new active cert is created; a unique index allows one active cert per user+type. The TC counted records regardless of status (revoked + active = 2) → false positive. Test fixed to count ACTIVE only + assert the renewal trail; TC 2060122 PASSES, be_gap removed.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="33.75" customFormat="1" customHeight="1" s="1">
       <c r="A4" s="7" t="inlineStr">
@@ -2848,213 +2856,209 @@
       </c>
     </row>
     <row r="33" ht="18.75" customHeight="1">
-      <c r="A33" s="7" t="n"/>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="7" t="n"/>
-      <c r="G33" s="7" t="n"/>
-      <c r="H33" s="7" t="n"/>
-      <c r="I33" s="7" t="n"/>
-      <c r="J33" s="7" t="n"/>
-      <c r="K33" s="7" t="n"/>
-      <c r="L33" s="7" t="n"/>
-      <c r="M33" s="7" t="n"/>
-      <c r="N33" s="7" t="n"/>
-      <c r="O33" s="7" t="n"/>
-      <c r="P33" s="7" t="n"/>
-    </row>
-    <row r="34" ht="18.75" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-031</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="n">
+        <v>2061402</v>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_TEAM_002</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_TEAM</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H33" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I33" s="15" t="inlineStr">
+        <is>
+          <t>Partner team directory read-by-id ignores the path parameter: a ghost (well-formed, absent) userId is not rejected, and a malformed userId is not rejected.</t>
+        </is>
+      </c>
+      <c r="J33" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/partner/directory/users/{userId}: a ghost (well-formed but non-existent) userId -&gt; 404 not found; a malformed userId -&gt; 400 invalid id.</t>
+        </is>
+      </c>
+      <c r="K33" s="15" t="inlineStr">
+        <is>
+          <t>ghost userId 000000000000000000000000 -&gt; HTTP 200 returning a DIFFERENT user (userId=6aba0a4b...); malformed userId 'not-an-id' -&gt; HTTP 200. The path parameter is ignored, so a caller reading a member it never asked for gets no error at all.</t>
+        </is>
+      </c>
+      <c r="L33" s="15" t="inlineStr">
+        <is>
+          <t>FAIL test_partner_api_partner_team_002 (run 2026-09-28): 'Validation gaps on /v1/partner/directory/users: ghost userId 000...000 returned HTTP 200 with userId=6aba0a4b... instead of 404; malformed userId not-an-id returned HTTP 200 instead of 400.'</t>
+        </is>
+      </c>
+      <c r="M33" s="15" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N33" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O33" s="15" t="n"/>
+      <c r="P33" s="15" t="inlineStr">
+        <is>
+          <t>Negative counterpart of BUG-API-022 (2061401) - SAME root cause: GET /directory/users/{userId} ignores the path param. Fix together with BUG-API-022/023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="204" customHeight="1">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>BUG-API-032</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="n">
+        <v>2061404</v>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_TEAM_004</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>PARTNER_TEAM</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H34" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I34" s="15" t="inlineStr">
+        <is>
+          <t>Team member deals/commissions read ignores the path parameter: a ghost/malformed userId is not rejected (reads as a member with no records).</t>
+        </is>
+      </c>
+      <c r="J34" s="15" t="inlineStr">
+        <is>
+          <t>GET /v1/partner/directory/users/{userId}/{deals,commissions}: a ghost userId -&gt; 404 not found; a malformed userId -&gt; 400 invalid id.</t>
+        </is>
+      </c>
+      <c r="K34" s="15" t="inlineStr">
+        <is>
+          <t>ghost userId -&gt; HTTP 200 with 0 rows (expected 404); malformed userId -&gt; HTTP 200 with 0 rows (expected 400). Path param ignored -&gt; a non-existent member reads as one that simply has no records; the same call returns ANOTHER member's deals when there ARE any (see BUG-API-023 / _003) = cross-member data disclosure risk.</t>
+        </is>
+      </c>
+      <c r="L34" s="15" t="inlineStr">
+        <is>
+          <t>FAIL test_partner_api_partner_team_004 (run 2026-09-28): 'Validation gaps on /v1/partner/directory/users/{userId}/{deals,commissions}: ghost userId answered 200 with 0 rows, expected 404 - the path parameter is ignored (BUG-API-023); malformed userId answered 200 with 0 rows, expected 400.'</t>
+        </is>
+      </c>
+      <c r="M34" s="15" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N34" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O34" s="15" t="n"/>
+      <c r="P34" s="15" t="inlineStr">
+        <is>
+          <t>Negative counterpart of BUG-API-023 (2061403) - SAME root cause: GET /directory/users/{userId}/{deals,commissions} ignores the path param. Fix together with BUG-API-022/023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18.75" customHeight="1">
+      <c r="A35" s="7" t="n"/>
+      <c r="B35" s="9" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="n"/>
+      <c r="H35" s="7" t="n"/>
+      <c r="I35" s="7" t="n"/>
+      <c r="J35" s="7" t="n"/>
+      <c r="K35" s="7" t="n"/>
+      <c r="L35" s="7" t="n"/>
+      <c r="M35" s="7" t="n"/>
+      <c r="N35" s="7" t="n"/>
+      <c r="O35" s="7" t="n"/>
+      <c r="P35" s="7" t="n"/>
+    </row>
+    <row r="36" ht="18.75" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="6" t="n"/>
-      <c r="J34" s="6" t="n"/>
-      <c r="K34" s="6" t="n"/>
-      <c r="L34" s="6" t="n"/>
-      <c r="M34" s="6" t="n"/>
-      <c r="N34" s="6" t="n"/>
-      <c r="O34" s="6" t="n"/>
-      <c r="P34" s="6" t="n"/>
-    </row>
-    <row r="35" ht="18.75" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>BUG-UI-001</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="n">
-        <v>12060101</v>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>PARTNER_UI_PARTNER_PORTAL_SHELL_001</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>PARTNER_PORTAL_SHELL</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>CLOSE</t>
-        </is>
-      </c>
-      <c r="I35" s="7" t="inlineStr">
-        <is>
-          <t>every primary nav page loads via URL (no MFE error).</t>
-        </is>
-      </c>
-      <c r="J35" s="7" t="inlineStr">
-        <is>
-          <t>every primary nav page loads via URL (no MFE error).</t>
-        </is>
-      </c>
-      <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="inlineStr">
-        <is>
-          <t>Page [apps] FAILED - Partner Portal section 'apps' rendered its shell but the CONTENT failed to load: banner 'Failed to load' is visible in &lt;main&gt;. Data-fetch/backend issue for this page — confirm with BE.</t>
-        </is>
-      </c>
-      <c r="M35" s="7" t="inlineStr">
-        <is>
-          <t>AI Triage</t>
-        </is>
-      </c>
-      <c r="N35" s="7" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-      <c r="O35" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="P35" s="7" t="inlineStr">
-        <is>
-          <t>CLOSED 2026-09-30 — no longer applicable: the 'My Apps' page was REMOVED from the partner portal (no nav item; /apps renders a 404 page). 'apps' dropped from the test; PARTNER_UI_PARTNER_PORTAL_SHELL_001 now PASSES 5/5, be_gap removed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18.75" customHeight="1">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>BUG-UI-002</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="n">
-        <v>12060102</v>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>PARTNER_UI_PARTNER_PORTAL_SHELL_002</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>PARTNER_PORTAL_SHELL</t>
-        </is>
-      </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H36" s="7" t="inlineStr">
-        <is>
-          <t>CLOSE</t>
-        </is>
-      </c>
-      <c r="I36" s="7" t="inlineStr">
-        <is>
-          <t>portal stays usable at mobile width (no h-overflow, nav reachable).</t>
-        </is>
-      </c>
-      <c r="J36" s="7" t="inlineStr">
-        <is>
-          <t>portal stays usable at mobile width (no h-overflow, nav reachable).</t>
-        </is>
-      </c>
-      <c r="K36" s="7" t="inlineStr">
-        <is>
-          <t>Page [deals] FAILED - 'deals' overflows the mobile viewport by 162px (content does not fit 375px → responsive-layout defect; confirm with FE)</t>
-        </is>
-      </c>
-      <c r="L36" s="7" t="inlineStr">
-        <is>
-          <t>Page [deals] FAILED - 'deals' overflows the mobile viewport by 162px (content does not fit 375px → responsive-layout defect; confirm with FE)</t>
-        </is>
-      </c>
-      <c r="M36" s="7" t="inlineStr">
-        <is>
-          <t>AI Triage</t>
-        </is>
-      </c>
-      <c r="N36" s="7" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="O36" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="P36" s="7" t="inlineStr">
-        <is>
-          <t>FIXED — re-verified 2026-09-30: /deals no longer overflows at 375px (was +162px). My Apps page removed from the portal. TC 12060102 still fails, but ONLY on /directory — a distinct defect logged as BUG-UI-010.</t>
-        </is>
-      </c>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="n"/>
+      <c r="I36" s="6" t="n"/>
+      <c r="J36" s="6" t="n"/>
+      <c r="K36" s="6" t="n"/>
+      <c r="L36" s="6" t="n"/>
+      <c r="M36" s="6" t="n"/>
+      <c r="N36" s="6" t="n"/>
+      <c r="O36" s="6" t="n"/>
+      <c r="P36" s="6" t="n"/>
     </row>
     <row r="37" ht="18.75" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>BUG-UI-003</t>
+          <t>BUG-UI-001</t>
         </is>
       </c>
       <c r="B37" s="9" t="n">
-        <v>12060203</v>
+        <v>12060101</v>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>PARTNER_UI_MY_PIPELINE_003</t>
+          <t>PARTNER_UI_PARTNER_PORTAL_SHELL_001</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -3064,7 +3068,7 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>MY_PIPELINE</t>
+          <t>PARTNER_PORTAL_SHELL</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
@@ -3084,22 +3088,18 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>an invalid domain must be rejected with a format error.</t>
+          <t>every primary nav page loads via URL (no MFE error).</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>an invalid domain must be rejected with a format error.</t>
-        </is>
-      </c>
-      <c r="K37" s="7" t="inlineStr">
-        <is>
-          <t>FAIL | [1/1] Each malformed domain must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts invalid domain(s) ["'@@@' (field kept '@@@', Next enabled, not flagged)", "'ab cd' (field kept 'ab cd', Next enabled, not flagged)</t>
-        </is>
-      </c>
+          <t>every primary nav page loads via URL (no MFE error).</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="n"/>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>FAIL | [1/1] Each malformed domain must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts invalid domain(s) ["'@@@' (field kept '@@@', Next enabled, not flagged)", "'ab cd' (field kept 'ab cd', Next enabled, not flagged)", "'notadomain' (field kept 'notadomain', Next en</t>
+          <t>Page [apps] FAILED - Partner Portal section 'apps' rendered its shell but the CONTENT failed to load: banner 'Failed to load' is visible in &lt;main&gt;. Data-fetch/backend issue for this page — confirm with BE.</t>
         </is>
       </c>
       <c r="M37" s="7" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="O37" s="7" t="inlineStr">
@@ -3119,231 +3119,239 @@
       </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>FIXED — re-verified 2026-09-30: the Domain field now validates ('Use letters, numbers, and hyphens only — no dots or symbols, e.g. my-company'). Test inputs corrected: 'notadomain' removed (VALID under the rule) and replaced with 'acme.com'. PARTNER_UI_MY_PIPELINE_003 PASSES, be_gap removed.</t>
+          <t>CLOSED 2026-09-30 — no longer applicable: the 'My Apps' page was REMOVED from the partner portal (no nav item; /apps renders a 404 page). 'apps' dropped from the test; PARTNER_UI_PARTNER_PORTAL_SHELL_001 now PASSES 5/5, be_gap removed.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18.75" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
         <is>
+          <t>BUG-UI-002</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="n">
+        <v>12060102</v>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>PARTNER_UI_PARTNER_PORTAL_SHELL_002</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>PARTNER_PORTAL_SHELL</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>portal stays usable at mobile width (no h-overflow, nav reachable).</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>portal stays usable at mobile width (no h-overflow, nav reachable).</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>Page [deals] FAILED - 'deals' overflows the mobile viewport by 162px (content does not fit 375px → responsive-layout defect; confirm with FE)</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t>Page [deals] FAILED - 'deals' overflows the mobile viewport by 162px (content does not fit 375px → responsive-layout defect; confirm with FE)</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N38" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="O38" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P38" s="7" t="inlineStr">
+        <is>
+          <t>FIXED — re-verified 2026-09-30: /deals no longer overflows at 375px (was +162px). My Apps page removed from the portal. TC 12060102 still fails, but ONLY on /directory — a distinct defect logged as BUG-UI-010.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18.75" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>BUG-UI-003</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="n">
+        <v>12060203</v>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>PARTNER_UI_MY_PIPELINE_003</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>MY_PIPELINE</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>an invalid domain must be rejected with a format error.</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>an invalid domain must be rejected with a format error.</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [1/1] Each malformed domain must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts invalid domain(s) ["'@@@' (field kept '@@@', Next enabled, not flagged)", "'ab cd' (field kept 'ab cd', Next enabled, not flagged)</t>
+        </is>
+      </c>
+      <c r="L39" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [1/1] Each malformed domain must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts invalid domain(s) ["'@@@' (field kept '@@@', Next enabled, not flagged)", "'ab cd' (field kept 'ab cd', Next enabled, not flagged)", "'notadomain' (field kept 'notadomain', Next en</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N39" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="O39" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P39" s="7" t="inlineStr">
+        <is>
+          <t>FIXED — re-verified 2026-09-30: the Domain field now validates ('Use letters, numbers, and hyphens only — no dots or symbols, e.g. my-company'). Test inputs corrected: 'notadomain' removed (VALID under the rule) and replaced with 'acme.com'. PARTNER_UI_MY_PIPELINE_003 PASSES, be_gap removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18.75" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
           <t>BUG-UI-004</t>
         </is>
       </c>
-      <c r="B38" s="9" t="n">
+      <c r="B40" s="9" t="n">
         <v>12060207</v>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>PARTNER_UI_MY_PIPELINE_007</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>MY_PIPELINE</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="H40" s="7" t="inlineStr">
         <is>
           <t>CLOSE
 CLOSE
 CLOSE</t>
         </is>
       </c>
-      <c r="I38" s="7" t="inlineStr">
+      <c r="I40" s="7" t="inlineStr">
         <is>
           <t>a malformed contact email must be rejected with a format error.</t>
         </is>
       </c>
-      <c r="J38" s="7" t="inlineStr">
+      <c r="J40" s="7" t="inlineStr">
         <is>
           <t>a malformed contact email must be rejected with a format error.</t>
         </is>
       </c>
-      <c r="K38" s="7" t="inlineStr">
+      <c r="K40" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">FAIL | [1/1] Each malformed email must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts malformed email(s) ["'notanemail' (field kept 'notanemail', Next enabled, not flagged)", "'abc@' (field kept 'abc@', Next enabled, </t>
         </is>
       </c>
-      <c r="L38" s="7" t="inlineStr">
+      <c r="L40" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">FAIL | [1/1] Each malformed email must be rejected (block Next / flag field) (246ms) -- AssertionError: wizard accepts malformed email(s) ["'notanemail' (field kept 'notanemail', Next enabled, not flagged)", "'abc@' (field kept 'abc@', Next enabled, not flagged)", "'abc@x' (field kept 'abc@x', Next </t>
         </is>
       </c>
-      <c r="M38" s="7" t="inlineStr">
+      <c r="M40" s="7" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N38" s="7" t="inlineStr">
+      <c r="N40" s="7" t="inlineStr">
         <is>
           <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="O38" s="7" t="n"/>
-      <c r="P38" s="7" t="n"/>
-    </row>
-    <row r="39" ht="18.75" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>BUG-UI-005</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="n">
-        <v>12060507</v>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>PARTNER_UI_SA_PARTNER_MODULE_007</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>SA_PARTNER_MODULE</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H39" s="7" t="inlineStr">
-        <is>
-          <t>CLOSE</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>SA Deal Approval Queue (/partners/deals): deal-list API consistently returns "Server Error - Invalid id: pro-v1" instead of the deals.</t>
-        </is>
-      </c>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>GET deal-list for /partners/deals returns the deals (200); the queue table shows deal rows. No "Invalid id" error.</t>
-        </is>
-      </c>
-      <c r="K39" s="7" t="inlineStr">
-        <is>
-          <t>The deal-list fetch consistently returns "Server Error - Invalid id: pro-v1"; the UI shows "No Data Found" and no deal rows load (partners DO have open deals).</t>
-        </is>
-      </c>
-      <c r="L39" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FAIL | [3/3] The Pending Approval + Conflicts queues load without a server error (3161ms) -- AssertionError: the deal approval queues must load their deals, but the deal-list fetch fails with a backend error on: ['Pending Approval: "Server Error Invalid id: \'pro-v1\' Server Error Invalid id: \'"', </t>
-        </is>
-      </c>
-      <c r="M39" s="7" t="inlineStr">
-        <is>
-          <t>AI Triage</t>
-        </is>
-      </c>
-      <c r="N39" s="7" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="O39" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="P39" s="7" t="inlineStr">
-        <is>
-          <t>FIXED — re-verified 2026-08-10: PARTNER_UI_SA_PARTNER_MODULE_007 now PASSES (15.3s, log: 'CHECK deals load -&gt; OK (no server error)'). The deal-list fetch no longer returns "Invalid id: 'pro-v1'". be_gap marker removed from the test and the registry re-synced, so this TC is back inside the merge gate. | Root cause = contract drift: a plan-slug "pro-v1" (string) is used where the API expects a Mongo _id (24-hex), so deal-list id validation fails. CONSISTENT, not intermittent (updated 2026-08-05): earlier "lucky PASS" runs were a TEST race - the assertion ran before the async deal-list error painted; the test now waits for the fetch to settle and fails deterministically. UI test 12060507 renders fine (shell/filters/headers OK); this step reflects the BE defect. Fix BE so deal-list never returns Invalid id: pro-v1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18.75" customHeight="1">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>BUG-UI-006</t>
-        </is>
-      </c>
-      <c r="B40" s="9" t="n">
-        <v>12060511</v>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>PARTNER_UI_SA_PARTNER_MODULE_011</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>SA_PARTNER_MODULE</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H40" s="7" t="inlineStr">
-        <is>
-          <t>CLOSE</t>
-        </is>
-      </c>
-      <c r="I40" s="7" t="inlineStr">
-        <is>
-          <t>the SA partner-programme analytics dashboard.</t>
-        </is>
-      </c>
-      <c r="J40" s="7" t="inlineStr">
-        <is>
-          <t>the SA partner-programme analytics dashboard.</t>
-        </is>
-      </c>
-      <c r="K40" s="7" t="inlineStr">
-        <is>
-          <t>FAIL | [3/3] The analytics data loads without a server error (44ms) -- AssertionError: the analytics dashboard must load its data, but a query fails with a backend error: 'Server Error limit must not be greater than 100 Server Error Invalid p'. The d</t>
-        </is>
-      </c>
-      <c r="L40" s="7" t="inlineStr">
-        <is>
-          <t>FAIL | [3/3] The analytics data loads without a server error (44ms) -- AssertionError: the analytics dashboard must load its data, but a query fails with a backend error: 'Server Error limit must not be greater than 100 Server Error Invalid p'. The dashboard shell renders but a paginated analytics q</t>
-        </is>
-      </c>
-      <c r="M40" s="7" t="inlineStr">
-        <is>
-          <t>AI Triage</t>
-        </is>
-      </c>
-      <c r="N40" s="7" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
         </is>
       </c>
       <c r="O40" s="7" t="n"/>
@@ -3352,15 +3360,15 @@
     <row r="41" ht="18.75" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>BUG-UI-007</t>
+          <t>BUG-UI-005</t>
         </is>
       </c>
       <c r="B41" s="9" t="n">
-        <v>12060405</v>
+        <v>12060507</v>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>PARTNER_UI_DASHBOARD_005</t>
+          <t>PARTNER_UI_SA_PARTNER_MODULE_007</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
@@ -3370,7 +3378,7 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>DASHBOARD</t>
+          <t>SA_PARTNER_MODULE</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
@@ -3385,27 +3393,27 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>CLOSE</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>tier-qualification math (T12M ARR threshold + next-tier delta).</t>
+          <t>SA Deal Approval Queue (/partners/deals): deal-list API consistently returns "Server Error - Invalid id: pro-v1" instead of the deals.</t>
         </is>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>tier-qualification math (T12M ARR threshold + next-tier delta).</t>
+          <t>GET deal-list for /partners/deals returns the deals (200); the queue table shows deal rows. No "Invalid id" error.</t>
         </is>
       </c>
       <c r="K41" s="7" t="inlineStr">
         <is>
-          <t>FAIL | [2/3] Next-tier T12M ARR threshold target + remaining delta are shown (0ms) -- AssertionError: the next-tier T12M ARR threshold target and remaining delta must be shown in Tier Progress, but only current tier/ARR/deal-count are rendered (panel</t>
+          <t>The deal-list fetch consistently returns "Server Error - Invalid id: pro-v1"; the UI shows "No Data Found" and no deal rows load (partners DO have open deals).</t>
         </is>
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>FAIL | [2/3] Next-tier T12M ARR threshold target + remaining delta are shown (0ms) -- AssertionError: the next-tier T12M ARR threshold target and remaining delta must be shown in Tier Progress, but only current tier/ARR/deal-count are rendered (panel='Tier &amp; Performance SELECT T12M ARR USD 0 Tier Pr</t>
+          <t xml:space="preserve">FAIL | [3/3] The Pending Approval + Conflicts queues load without a server error (3161ms) -- AssertionError: the deal approval queues must load their deals, but the deal-list fetch fails with a backend error on: ['Pending Approval: "Server Error Invalid id: \'pro-v1\' Server Error Invalid id: \'"', </t>
         </is>
       </c>
       <c r="M41" s="7" t="inlineStr">
@@ -3415,260 +3423,256 @@
       </c>
       <c r="N41" s="7" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="O41" s="7" t="n"/>
-      <c r="P41" s="7" t="n"/>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="O41" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="P41" s="7" t="inlineStr">
+        <is>
+          <t>FIXED — re-verified 2026-08-10: PARTNER_UI_SA_PARTNER_MODULE_007 now PASSES (15.3s, log: 'CHECK deals load -&gt; OK (no server error)'). The deal-list fetch no longer returns "Invalid id: 'pro-v1'". be_gap marker removed from the test and the registry re-synced, so this TC is back inside the merge gate. | Root cause = contract drift: a plan-slug "pro-v1" (string) is used where the API expects a Mongo _id (24-hex), so deal-list id validation fails. CONSISTENT, not intermittent (updated 2026-08-05): earlier "lucky PASS" runs were a TEST race - the assertion ran before the async deal-list error painted; the test now waits for the fetch to settle and fails deterministically. UI test 12060507 renders fine (shell/filters/headers OK); this step reflects the BE defect. Fix BE so deal-list never returns Invalid id: pro-v1.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18.75" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
+          <t>BUG-UI-006</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>12060511</v>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>PARTNER_UI_SA_PARTNER_MODULE_011</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>SA_PARTNER_MODULE</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>the SA partner-programme analytics dashboard.</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>the SA partner-programme analytics dashboard.</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [3/3] The analytics data loads without a server error (44ms) -- AssertionError: the analytics dashboard must load its data, but a query fails with a backend error: 'Server Error limit must not be greater than 100 Server Error Invalid p'. The d</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [3/3] The analytics data loads without a server error (44ms) -- AssertionError: the analytics dashboard must load its data, but a query fails with a backend error: 'Server Error limit must not be greater than 100 Server Error Invalid p'. The dashboard shell renders but a paginated analytics q</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N42" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="O42" s="7" t="n"/>
+      <c r="P42" s="7" t="n"/>
+    </row>
+    <row r="43" ht="18.75" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>BUG-UI-007</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>12060405</v>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>PARTNER_UI_DASHBOARD_005</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>DASHBOARD</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>tier-qualification math (T12M ARR threshold + next-tier delta).</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>tier-qualification math (T12M ARR threshold + next-tier delta).</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [2/3] Next-tier T12M ARR threshold target + remaining delta are shown (0ms) -- AssertionError: the next-tier T12M ARR threshold target and remaining delta must be shown in Tier Progress, but only current tier/ARR/deal-count are rendered (panel</t>
+        </is>
+      </c>
+      <c r="L43" s="7" t="inlineStr">
+        <is>
+          <t>FAIL | [2/3] Next-tier T12M ARR threshold target + remaining delta are shown (0ms) -- AssertionError: the next-tier T12M ARR threshold target and remaining delta must be shown in Tier Progress, but only current tier/ARR/deal-count are rendered (panel='Tier &amp; Performance SELECT T12M ARR USD 0 Tier Pr</t>
+        </is>
+      </c>
+      <c r="M43" s="7" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="O43" s="7" t="n"/>
+      <c r="P43" s="7" t="n"/>
+    </row>
+    <row r="44" ht="18.75" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
           <t>BUG-UI-008</t>
         </is>
       </c>
-      <c r="B42" s="9" t="n">
+      <c r="B44" s="9" t="n">
         <v>12060515</v>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C44" s="7" t="inlineStr">
         <is>
           <t>PARTNER_UI_SA_PARTNER_MODULE_015</t>
         </is>
       </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
         <is>
           <t>SA_PARTNER_MODULE</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G44" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H44" s="7" t="inlineStr">
         <is>
           <t>CLOSE</t>
         </is>
       </c>
-      <c r="I42" s="7" t="inlineStr">
+      <c r="I44" s="7" t="inlineStr">
         <is>
           <t>suspend (deactivate) an active partner.</t>
         </is>
       </c>
-      <c r="J42" s="7" t="inlineStr">
+      <c r="J44" s="7" t="inlineStr">
         <is>
           <t>SA can suspend an Active partner from Partner Detail -&gt; Partner actions -&gt; Deactivate: partner transitions to Suspended/Inactive and loses portal access.</t>
         </is>
       </c>
-      <c r="K42" s="7" t="inlineStr">
+      <c r="K44" s="7" t="inlineStr">
         <is>
           <t>Deactivate fails. The "Deactivate Partner" confirm dialog collects NO reason, so the FE calls the deactivate API without one; BE returns 400 Server Error ("reason should not be empty / reason must be a string / reason must be &lt;= 2000 characters"). Partner stays Active. No SA can suspend a partner via the UI.</t>
         </is>
       </c>
-      <c r="L42" s="7" t="inlineStr">
+      <c r="L44" s="7" t="inlineStr">
         <is>
           <t>FAIL | [2/2] The partner is suspended and no error is shown (0ms) -- AssertionError: Deactivate failed — the BE rejected the request: 'Failed to deactivate partner Server Error reason must be shorter than or equal to 2000 charactersreason should not be emptyreason must be a string Partner approved Q</t>
         </is>
       </c>
-      <c r="M42" s="7" t="inlineStr">
+      <c r="M44" s="7" t="inlineStr">
         <is>
           <t>AI Triage</t>
         </is>
       </c>
-      <c r="N42" s="7" t="inlineStr">
+      <c r="N44" s="7" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="O42" s="7" t="inlineStr">
+      <c r="O44" s="7" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="P42" s="7" t="inlineStr">
+      <c r="P44" s="7" t="inlineStr">
         <is>
           <t>FIXED — re-verified 2026-09-30: the Deactivate Partner dialog now has a required Reason textarea (Deactivate disabled until filled); the request succeeds and the partner becomes Suspended. PARTNER_UI_SA_PARTNER_MODULE_015 PASSES, be_gap removed. Unblocks _016 (reactivate). | FE&lt;-&gt;BE contract mismatch. Fix options: (a) add a required Reason textarea to the Deactivate dialog and send it, or (b) make reason optional on the deactivate API. Repro: onboard partner -&gt; Approve -&gt; Partner actions -&gt; Deactivate -&gt; Confirm. Blocks SA_PARTNER_MODULE_016 (reactivate) too. TC marked be_gap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="18.75" customHeight="1">
-      <c r="A43" s="15" t="inlineStr">
-        <is>
-          <t>BUG-UI-009</t>
-        </is>
-      </c>
-      <c r="B43" s="14" t="n">
-        <v>12060201</v>
-      </c>
-      <c r="C43" s="15" t="inlineStr">
-        <is>
-          <t>PARTNER_UI_MY_PIPELINE_001</t>
-        </is>
-      </c>
-      <c r="D43" s="15" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E43" s="15" t="inlineStr">
-        <is>
-          <t>MY_PIPELINE</t>
-        </is>
-      </c>
-      <c r="F43" s="15" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G43" s="15" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="H43" s="15" t="inlineStr">
-        <is>
-          <t>CLOSE</t>
-        </is>
-      </c>
-      <c r="I43" s="15" t="inlineStr">
-        <is>
-          <t>Register-a-Deal wizard: Country dropdown is empty ('No options') on Chrome/Chromium (works on Edge). The wizard's countries lookup is sent WITHOUT an Authorization header -&gt; 401, so no country can be selected and a deal cannot be registered.</t>
-        </is>
-      </c>
-      <c r="J43" s="15" t="inlineStr">
-        <is>
-          <t>On every browser (incl. Chrome) the Country dropdown lists countries; partner completes Step 1 and registers a deal.</t>
-        </is>
-      </c>
-      <c r="K43" s="15" t="inlineStr">
-        <is>
-          <t>On Chrome/Chromium (manual AND automation), GET /sa-partners-api/v1/partner/portal/countries is sent with NO Authorization header -&gt; 401 -&gt; dropdown shows 'No options' -&gt; Step 1 cannot be completed. On Edge (manual) the same request carries the bearer token -&gt; 200 -&gt; options load.</t>
-        </is>
-      </c>
-      <c r="L43" s="15" t="inlineStr">
-        <is>
-          <t>countries request hasAuth=false -&gt; 401 on Chromium (Playwright) and manual Chrome; 200 on manual Edge. Shell /partner/auth/refresh + /auth/me return 200, so the shell is authenticated but the token is not attached to the MFE's countries call. Manual repro: Chrome FAIL / Edge PASS.</t>
-        </is>
-      </c>
-      <c r="M43" s="15" t="inlineStr">
-        <is>
-          <t>tam.do@terralogic.com</t>
-        </is>
-      </c>
-      <c r="N43" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="O43" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="P43" s="15" t="inlineStr">
-        <is>
-          <t>FIXED — verified manually by QA on 2026-09-30 (ticket BLAZ7-5-27 PV VALIDATION → CLOSED): Country dropdown loads on Chrome. | Browser-specific (Chrome/Chromium FAIL, Edge PASS) at BOTH manual and automation level. Affects all 11 register-wizard TCs: 12060201-12060208, 12060211-12060213 (automation runs on Chromium -&gt; all fail). Leading hypothesis for FE: Chrome's stricter storage-partitioning / third-party-context defaults block the deals micro-frontend (partnerDealsApp, which has its own token-store bundle) from reading the auth token (pp_refresh_token in sessionStorage) -&gt; token not attached to the countries request. FE to verify how partnerDealsApp obtains/attaches the access token on Chrome. NOTE: AI triage mislabels these as [FLAKY] (Locator.click-timeout heuristic) - they are deterministic, not flaky.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18.75" customHeight="1">
-      <c r="A44" s="15" t="inlineStr">
-        <is>
-          <t>BUG-API-031</t>
-        </is>
-      </c>
-      <c r="B44" s="14" t="n">
-        <v>2061402</v>
-      </c>
-      <c r="C44" s="15" t="inlineStr">
-        <is>
-          <t>PARTNER_API_PARTNER_TEAM_002</t>
-        </is>
-      </c>
-      <c r="D44" s="15" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E44" s="15" t="inlineStr">
-        <is>
-          <t>PARTNER_TEAM</t>
-        </is>
-      </c>
-      <c r="F44" s="15" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="G44" s="15" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H44" s="15" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I44" s="15" t="inlineStr">
-        <is>
-          <t>Partner team directory read-by-id ignores the path parameter: a ghost (well-formed, absent) userId is not rejected, and a malformed userId is not rejected.</t>
-        </is>
-      </c>
-      <c r="J44" s="15" t="inlineStr">
-        <is>
-          <t>GET /v1/partner/directory/users/{userId}: a ghost (well-formed but non-existent) userId -&gt; 404 not found; a malformed userId -&gt; 400 invalid id.</t>
-        </is>
-      </c>
-      <c r="K44" s="15" t="inlineStr">
-        <is>
-          <t>ghost userId 000000000000000000000000 -&gt; HTTP 200 returning a DIFFERENT user (userId=6aba0a4b...); malformed userId 'not-an-id' -&gt; HTTP 200. The path parameter is ignored, so a caller reading a member it never asked for gets no error at all.</t>
-        </is>
-      </c>
-      <c r="L44" s="15" t="inlineStr">
-        <is>
-          <t>FAIL test_partner_api_partner_team_002 (run 2026-09-28): 'Validation gaps on /v1/partner/directory/users: ghost userId 000...000 returned HTTP 200 with userId=6aba0a4b... instead of 404; malformed userId not-an-id returned HTTP 200 instead of 400.'</t>
-        </is>
-      </c>
-      <c r="M44" s="15" t="inlineStr">
-        <is>
-          <t>AI Triage</t>
-        </is>
-      </c>
-      <c r="N44" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="O44" s="15" t="n"/>
-      <c r="P44" s="15" t="inlineStr">
-        <is>
-          <t>Negative counterpart of BUG-API-022 (2061401) - SAME root cause: GET /directory/users/{userId} ignores the path param. Fix together with BUG-API-022/023.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="204" customHeight="1">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t>BUG-API-032</t>
+          <t>BUG-UI-009</t>
         </is>
       </c>
       <c r="B45" s="14" t="n">
-        <v>2061404</v>
+        <v>12060201</v>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>PARTNER_API_PARTNER_TEAM_004</t>
+          <t>PARTNER_UI_MY_PIPELINE_001</t>
         </is>
       </c>
       <c r="D45" s="15" t="inlineStr">
@@ -3678,47 +3682,47 @@
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>PARTNER_TEAM</t>
+          <t>MY_PIPELINE</t>
         </is>
       </c>
       <c r="F45" s="15" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G45" s="15" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H45" s="15" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>CLOSE</t>
         </is>
       </c>
       <c r="I45" s="15" t="inlineStr">
         <is>
-          <t>Team member deals/commissions read ignores the path parameter: a ghost/malformed userId is not rejected (reads as a member with no records).</t>
+          <t>Register-a-Deal wizard: Country dropdown is empty ('No options') on Chrome/Chromium (works on Edge). The wizard's countries lookup is sent WITHOUT an Authorization header -&gt; 401, so no country can be selected and a deal cannot be registered.</t>
         </is>
       </c>
       <c r="J45" s="15" t="inlineStr">
         <is>
-          <t>GET /v1/partner/directory/users/{userId}/{deals,commissions}: a ghost userId -&gt; 404 not found; a malformed userId -&gt; 400 invalid id.</t>
+          <t>On every browser (incl. Chrome) the Country dropdown lists countries; partner completes Step 1 and registers a deal.</t>
         </is>
       </c>
       <c r="K45" s="15" t="inlineStr">
         <is>
-          <t>ghost userId -&gt; HTTP 200 with 0 rows (expected 404); malformed userId -&gt; HTTP 200 with 0 rows (expected 400). Path param ignored -&gt; a non-existent member reads as one that simply has no records; the same call returns ANOTHER member's deals when there ARE any (see BUG-API-023 / _003) = cross-member data disclosure risk.</t>
+          <t>On Chrome/Chromium (manual AND automation), GET /sa-partners-api/v1/partner/portal/countries is sent with NO Authorization header -&gt; 401 -&gt; dropdown shows 'No options' -&gt; Step 1 cannot be completed. On Edge (manual) the same request carries the bearer token -&gt; 200 -&gt; options load.</t>
         </is>
       </c>
       <c r="L45" s="15" t="inlineStr">
         <is>
-          <t>FAIL test_partner_api_partner_team_004 (run 2026-09-28): 'Validation gaps on /v1/partner/directory/users/{userId}/{deals,commissions}: ghost userId answered 200 with 0 rows, expected 404 - the path parameter is ignored (BUG-API-023); malformed userId answered 200 with 0 rows, expected 400.'</t>
+          <t>countries request hasAuth=false -&gt; 401 on Chromium (Playwright) and manual Chrome; 200 on manual Edge. Shell /partner/auth/refresh + /auth/me return 200, so the shell is authenticated but the token is not attached to the MFE's countries call. Manual repro: Chrome FAIL / Edge PASS.</t>
         </is>
       </c>
       <c r="M45" s="15" t="inlineStr">
         <is>
-          <t>AI Triage</t>
+          <t>tam.do@terralogic.com</t>
         </is>
       </c>
       <c r="N45" s="15" t="inlineStr">
@@ -3726,10 +3730,14 @@
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="O45" s="15" t="n"/>
+      <c r="O45" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="P45" s="15" t="inlineStr">
         <is>
-          <t>Negative counterpart of BUG-API-023 (2061403) - SAME root cause: GET /directory/users/{userId}/{deals,commissions} ignores the path param. Fix together with BUG-API-022/023.</t>
+          <t>FIXED — verified manually by QA on 2026-09-30 (ticket BLAZ7-5-27 PV VALIDATION → CLOSED): Country dropdown loads on Chrome. | Browser-specific (Chrome/Chromium FAIL, Edge PASS) at BOTH manual and automation level. Affects all 11 register-wizard TCs: 12060201-12060208, 12060211-12060213 (automation runs on Chromium -&gt; all fail). Leading hypothesis for FE: Chrome's stricter storage-partitioning / third-party-context defaults block the deals micro-frontend (partnerDealsApp, which has its own token-store bundle) from reading the auth token (pp_refresh_token in sessionStorage) -&gt; token not attached to the countries request. FE to verify how partnerDealsApp obtains/attaches the access token on Chrome. NOTE: AI triage mislabels these as [FLAKY] (Locator.click-timeout heuristic) - they are deterministic, not flaky.</t>
         </is>
       </c>
     </row>

</xml_diff>